<commit_message>
Att Chamada 1A 15-09
</commit_message>
<xml_diff>
--- a/ds/turmas/1DES_A/frequencia-2-A.xlsx
+++ b/ds/turmas/1DES_A/frequencia-2-A.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sn1089986\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sn1053361\Documents\senai2026\ds\turmas\1DES_A\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC5F2CE6-DBB3-4AF5-8155-C3F9E189480C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{229DF955-1E70-4201-8696-5E49D8BF6E96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1965" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1966" uniqueCount="53">
   <si>
     <t>Aluno</t>
   </si>
@@ -195,6 +195,9 @@
   <si>
     <t>5P|F</t>
   </si>
+  <si>
+    <t>P | 5F</t>
+  </si>
 </sst>
 </file>
 
@@ -279,7 +282,87 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="15">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -827,7 +910,9 @@
       <c r="BH1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="BI1" s="1"/>
+      <c r="BI1" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="BJ1" s="1"/>
       <c r="BK1" s="1"/>
       <c r="BL1" s="1"/>
@@ -1041,7 +1126,9 @@
       <c r="BH2" s="1">
         <v>46275</v>
       </c>
-      <c r="BI2" s="1"/>
+      <c r="BI2" s="1">
+        <v>46280</v>
+      </c>
       <c r="BJ2" s="1"/>
       <c r="BK2" s="1"/>
       <c r="BL2" s="1"/>
@@ -4713,7 +4800,7 @@
         <v>31</v>
       </c>
       <c r="BI17" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="BJ17" s="3"/>
       <c r="BK17" s="3"/>
@@ -5439,7 +5526,7 @@
         <v>31</v>
       </c>
       <c r="BI20" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="BJ20" s="3"/>
       <c r="BK20" s="3"/>
@@ -7920,7 +8007,7 @@
         <v>31</v>
       </c>
       <c r="BI30" s="3" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="BJ30" s="3"/>
       <c r="BK30" s="3"/>
@@ -8740,38 +8827,43 @@
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="G31:I32">
-    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="9" operator="equal">
       <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U3:AS34">
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="7" operator="equal">
       <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AU3:BA3 BF3:DH3 BC3:BC21 D3:I30 K3:T30 AZ4:BA9 BF4:BF9 AU4:AY26 BH4:BH30 BG4:BG34 AZ10:BB21 BD10:BF21 AZ22:BF26 AU27:BF28 AU29:AX30 AZ29:BF30 AY29:AY34 K31:K33 L31:T34 AU31:AV34 H33:I33 BJ4:DH30 BI4:BI34">
-    <cfRule type="cellIs" dxfId="4" priority="10" operator="equal">
+  <conditionalFormatting sqref="AU3:BA3 BF3:DH3 BC3:BC21 D3:I30 K3:T30 AZ4:BA9 BF4:BF9 AU4:AY26 BH4:BH30 BJ4:DH30 BG4:BG34 BI4:BI34 AZ10:BB21 BD10:BF21 AZ22:BF26 AU27:BF28 AU29:AX30 AZ29:BF30 AY29:AY34 K31:K33 L31:T34 AU31:AV34 H33:I33">
+    <cfRule type="cellIs" dxfId="12" priority="11" operator="equal">
       <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BB9">
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="6" operator="equal">
       <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BB32">
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="5" operator="equal">
       <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BD3:BD34">
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="F">
+    <cfRule type="containsText" dxfId="9" priority="4" operator="containsText" text="F">
       <formula>NOT(ISERROR(SEARCH("F",BD3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BH3:BH34">
+    <cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="F">
+      <formula>NOT(ISERROR(SEARCH("F",BH3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BI3:BI34">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="F">
-      <formula>NOT(ISERROR(SEARCH("F",BH3)))</formula>
+      <formula>NOT(ISERROR(SEARCH("F",BI3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>